<commit_message>
Add Sphinx Qwen7B final20 eval results
</commit_message>
<xml_diff>
--- a/results/trace_final20_temp06_3b7b_model_results.xlsx
+++ b/results/trace_final20_temp06_3b7b_model_results.xlsx
@@ -10,7 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3B" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7B" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'3B'!$A$1:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'7B'!$A$1:$F$22</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +32,27 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -56,12 +73,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,34 +453,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Benchmark</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Rows</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Qwen2.5-VL-3B Base (3-seed avg)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Qwen2.5-VL-3B Answer GRPO 500 (3-seed avg)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Qwen2.5-VL-3B Annotation GRPO 500 (seed42)</t>
         </is>
@@ -473,13 +495,13 @@
       <c r="B2" t="n">
         <v>1901</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>44.52</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>46.5</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>47.02788006312467</v>
       </c>
     </row>
@@ -492,13 +514,13 @@
       <c r="B3" t="n">
         <v>1000</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>17.83</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>21.3</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>18</v>
       </c>
     </row>
@@ -511,13 +533,13 @@
       <c r="B4" t="n">
         <v>1948</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>32.08</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>33.27</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>33.81667309415904</v>
       </c>
     </row>
@@ -530,13 +552,13 @@
       <c r="B5" t="n">
         <v>1000</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>29.2</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>34.27</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>32.7</v>
       </c>
     </row>
@@ -549,13 +571,13 @@
       <c r="B6" t="n">
         <v>487</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>65.56999999999999</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>68.65000000000001</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>73.30595482546201</v>
       </c>
     </row>
@@ -568,13 +590,13 @@
       <c r="B7" t="n">
         <v>1200</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="3" t="n">
         <v>59.5</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>67.31</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>62.58333333333334</v>
       </c>
     </row>
@@ -587,13 +609,13 @@
       <c r="B8" t="n">
         <v>2633</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="3" t="n">
         <v>18.6</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>20.96</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>21.30649449297379</v>
       </c>
     </row>
@@ -606,13 +628,13 @@
       <c r="B9" t="n">
         <v>447</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="3" t="n">
         <v>36.84</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>42.65</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>36.46532438478747</v>
       </c>
     </row>
@@ -625,13 +647,13 @@
       <c r="B10" t="n">
         <v>3040</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="3" t="n">
         <v>19.93</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="3" t="n">
         <v>24.61</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>21.875</v>
       </c>
     </row>
@@ -644,13 +666,13 @@
       <c r="B11" t="n">
         <v>1000</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="3" t="n">
         <v>58.43</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>64.59999999999999</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" t="n">
         <v>64</v>
       </c>
     </row>
@@ -663,13 +685,13 @@
       <c r="B12" t="n">
         <v>1730</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="3" t="n">
         <v>26.76</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="3" t="n">
         <v>30.83</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>27.6878612716763</v>
       </c>
     </row>
@@ -682,13 +704,13 @@
       <c r="B13" t="n">
         <v>1297</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="3" t="n">
         <v>20.59</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="3" t="n">
         <v>20.43</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="3" t="n">
         <v>20.20046260601388</v>
       </c>
     </row>
@@ -701,13 +723,13 @@
       <c r="B14" t="n">
         <v>1000</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="3" t="n">
         <v>32.97</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <v>37.73</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>33.8</v>
       </c>
     </row>
@@ -720,13 +742,13 @@
       <c r="B15" t="n">
         <v>2000</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="3" t="n">
         <v>33.03</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="3" t="n">
         <v>40.35</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>37.85</v>
       </c>
     </row>
@@ -739,13 +761,13 @@
       <c r="B16" t="n">
         <v>1272</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="3" t="n">
         <v>60.51</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="3" t="n">
         <v>58.75</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>63.4433962264151</v>
       </c>
     </row>
@@ -758,13 +780,13 @@
       <c r="B17" t="n">
         <v>1180</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C17" s="3" t="n">
         <v>25.45</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="3" t="n">
         <v>26.86</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="3" t="n">
         <v>28.13559322033898</v>
       </c>
     </row>
@@ -777,13 +799,13 @@
       <c r="B18" t="n">
         <v>1500</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="3" t="n">
         <v>69.12</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="3" t="n">
         <v>71.88</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="3" t="n">
         <v>72.48</v>
       </c>
     </row>
@@ -796,13 +818,13 @@
       <c r="B19" t="n">
         <v>405</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="3" t="n">
         <v>39.18</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="3" t="n">
         <v>40.74</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="3" t="n">
         <v>38.2716049382716</v>
       </c>
     </row>
@@ -815,13 +837,13 @@
       <c r="B20" t="n">
         <v>1168</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="3" t="n">
         <v>17.32</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="3" t="n">
         <v>18.86</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="3" t="n">
         <v>17.38013698630137</v>
       </c>
     </row>
@@ -834,34 +856,35 @@
       <c r="B21" t="n">
         <v>1740</v>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="3" t="n">
         <v>46.93</v>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="3" t="n">
         <v>57.87</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="3" t="n">
         <v>51.66666666666667</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" s="2" t="n">
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="5" t="n">
         <v>37.718</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="5" t="n">
         <v>41.421</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="5" t="n">
         <v>40.09981910547621</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -872,40 +895,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Benchmark</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Rows</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Qwen2.5-VL-7B Base (3-seed avg)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Qwen2.5-VL-7B Answer GRPO 500 (3-seed avg)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>OpenMOSS Game-RL Qwen2.5-VL-7B (seed42)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Sphinx Qwen2.5-VL-7B 500 (seed42)</t>
         </is>
       </c>
     </row>
@@ -918,14 +947,17 @@
       <c r="B2" t="n">
         <v>1901</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>53.2</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>58.76</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>54.07680168332457</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>55.33929510783798</v>
       </c>
     </row>
     <row r="3">
@@ -937,14 +969,17 @@
       <c r="B3" t="n">
         <v>1000</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>24.43</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>32.5</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>24.5</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>24.4</v>
       </c>
     </row>
     <row r="4">
@@ -956,14 +991,17 @@
       <c r="B4" t="n">
         <v>1948</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>46.55</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>49.03</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>46.85464637181915</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>44.68253819100296</v>
       </c>
     </row>
     <row r="5">
@@ -975,14 +1013,17 @@
       <c r="B5" t="n">
         <v>1000</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>39.17</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>46.43</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>39.7</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>40.6</v>
       </c>
     </row>
     <row r="6">
@@ -994,14 +1035,17 @@
       <c r="B6" t="n">
         <v>487</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>82.81999999999999</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>85.08</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>84.80492813141683</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>83.16221765913757</v>
       </c>
     </row>
     <row r="7">
@@ -1013,14 +1057,17 @@
       <c r="B7" t="n">
         <v>1200</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="3" t="n">
         <v>76.67</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>81.39</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>75.83333333333333</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>79.91666666666667</v>
       </c>
     </row>
     <row r="8">
@@ -1032,14 +1079,17 @@
       <c r="B8" t="n">
         <v>2633</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="3" t="n">
         <v>24.93</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>29.08</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>30.26965438663122</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>25.06646410938094</v>
       </c>
     </row>
     <row r="9">
@@ -1051,14 +1101,17 @@
       <c r="B9" t="n">
         <v>447</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="3" t="n">
         <v>42.8</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>47.73</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>44.07158836689038</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>43.40044742729307</v>
       </c>
     </row>
     <row r="10">
@@ -1070,14 +1123,17 @@
       <c r="B10" t="n">
         <v>3040</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="3" t="n">
         <v>25.96</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="3" t="n">
         <v>27.96</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>26.48026315789473</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>26.28289473684211</v>
       </c>
     </row>
     <row r="11">
@@ -1089,14 +1145,17 @@
       <c r="B11" t="n">
         <v>1000</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="3" t="n">
         <v>69.13</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>73.43000000000001</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" t="n">
         <v>68</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>70.8</v>
       </c>
     </row>
     <row r="12">
@@ -1108,14 +1167,17 @@
       <c r="B12" t="n">
         <v>1730</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="3" t="n">
         <v>35.03</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="3" t="n">
         <v>39.88</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>35.83815028901734</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>36.99421965317919</v>
       </c>
     </row>
     <row r="13">
@@ -1127,14 +1189,17 @@
       <c r="B13" t="n">
         <v>1297</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="3" t="n">
         <v>20.71</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="3" t="n">
         <v>25.8</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="3" t="n">
         <v>21.04857363145721</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>20.35466461063994</v>
       </c>
     </row>
     <row r="14">
@@ -1146,14 +1211,17 @@
       <c r="B14" t="n">
         <v>1000</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="3" t="n">
         <v>40.1</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <v>47.63</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>40.40000000000001</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>40.9</v>
       </c>
     </row>
     <row r="15">
@@ -1165,14 +1233,17 @@
       <c r="B15" t="n">
         <v>2000</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="3" t="n">
         <v>46.85</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="3" t="n">
         <v>53.18</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>49.45</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>47.15</v>
       </c>
     </row>
     <row r="16">
@@ -1184,14 +1255,17 @@
       <c r="B16" t="n">
         <v>1272</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="3" t="n">
         <v>72.8</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="3" t="n">
         <v>77.73</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>75.23584905660378</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>81.05345911949685</v>
       </c>
     </row>
     <row r="17">
@@ -1203,14 +1277,17 @@
       <c r="B17" t="n">
         <v>1180</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C17" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="3" t="n">
         <v>31.61</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="3" t="n">
         <v>29.40677966101695</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>27.88135593220339</v>
       </c>
     </row>
     <row r="18">
@@ -1222,14 +1299,17 @@
       <c r="B18" t="n">
         <v>1500</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="3" t="n">
         <v>74.92</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="3" t="n">
         <v>77.98999999999999</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="3" t="n">
         <v>74.1333334</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>73.11999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -1241,14 +1321,17 @@
       <c r="B19" t="n">
         <v>405</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="3" t="n">
         <v>40.91</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="3" t="n">
         <v>43.21</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="3" t="n">
         <v>39.25925925925926</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>40.49382716049383</v>
       </c>
     </row>
     <row r="20">
@@ -1260,14 +1343,17 @@
       <c r="B20" t="n">
         <v>1168</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="3" t="n">
         <v>19.35</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="3" t="n">
         <v>22.32</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="3" t="n">
         <v>19.17808219178082</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>18.49315068493151</v>
       </c>
     </row>
     <row r="21">
@@ -1279,34 +1365,41 @@
       <c r="B21" t="n">
         <v>1740</v>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="3" t="n">
         <v>63.95</v>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="3" t="n">
         <v>67.89</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="3" t="n">
         <v>65.3448275862069</v>
       </c>
+      <c r="F21" s="3" t="n">
+        <v>65.17241379310344</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" s="2" t="n">
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="5" t="n">
         <v>46.339</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="5" t="n">
         <v>50.9315</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="5" t="n">
         <v>47.19430352533262</v>
       </c>
+      <c r="F22" s="5" t="n">
+        <v>47.26318074261048</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add PCGRPO Qwen7B final20 eval results
</commit_message>
<xml_diff>
--- a/results/trace_final20_temp06_3b7b_model_results.xlsx
+++ b/results/trace_final20_temp06_3b7b_model_results.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'3B'!$A$1:$E$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'7B'!$A$1:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'7B'!$A$1:$G$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,8 +455,8 @@
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -895,15 +895,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -937,6 +938,11 @@
           <t>Sphinx Qwen2.5-VL-7B 500 (seed42)</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>PCGRPO Qwen2.5-VL-7B Jigsaw CARE (seed42)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -959,6 +965,9 @@
       <c r="F2" s="3" t="n">
         <v>55.33929510783798</v>
       </c>
+      <c r="G2" s="3" t="n">
+        <v>56.23356128353498</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -981,6 +990,9 @@
       <c r="F3" s="3" t="n">
         <v>24.4</v>
       </c>
+      <c r="G3" s="3" t="n">
+        <v>25.1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1003,6 +1015,9 @@
       <c r="F4" s="3" t="n">
         <v>44.68253819100296</v>
       </c>
+      <c r="G4" s="3" t="n">
+        <v>41.27010074437245</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1025,6 +1040,9 @@
       <c r="F5" s="3" t="n">
         <v>40.6</v>
       </c>
+      <c r="G5" s="3" t="n">
+        <v>40.8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1047,6 +1065,9 @@
       <c r="F6" s="3" t="n">
         <v>83.16221765913757</v>
       </c>
+      <c r="G6" s="3" t="n">
+        <v>82.95687885010267</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1069,6 +1090,9 @@
       <c r="F7" s="3" t="n">
         <v>79.91666666666667</v>
       </c>
+      <c r="G7" s="3" t="n">
+        <v>81.08333333333333</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1091,6 +1115,9 @@
       <c r="F8" s="3" t="n">
         <v>25.06646410938094</v>
       </c>
+      <c r="G8" s="3" t="n">
+        <v>25.93999240410179</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1113,6 +1140,9 @@
       <c r="F9" s="3" t="n">
         <v>43.40044742729307</v>
       </c>
+      <c r="G9" s="3" t="n">
+        <v>43.17673378076063</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1135,6 +1165,9 @@
       <c r="F10" s="3" t="n">
         <v>26.28289473684211</v>
       </c>
+      <c r="G10" s="3" t="n">
+        <v>25.39473684210526</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1157,6 +1190,9 @@
       <c r="F11" s="3" t="n">
         <v>70.8</v>
       </c>
+      <c r="G11" s="3" t="n">
+        <v>71.09999999999999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1179,6 +1215,9 @@
       <c r="F12" s="3" t="n">
         <v>36.99421965317919</v>
       </c>
+      <c r="G12" s="3" t="n">
+        <v>34.27745664739884</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1201,6 +1240,9 @@
       <c r="F13" s="3" t="n">
         <v>20.35466461063994</v>
       </c>
+      <c r="G13" s="3" t="n">
+        <v>16.73091750192753</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1223,6 +1265,9 @@
       <c r="F14" s="3" t="n">
         <v>40.9</v>
       </c>
+      <c r="G14" s="3" t="n">
+        <v>42.7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1245,6 +1290,9 @@
       <c r="F15" s="3" t="n">
         <v>47.15</v>
       </c>
+      <c r="G15" s="3" t="n">
+        <v>50.05</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1267,6 +1315,9 @@
       <c r="F16" s="3" t="n">
         <v>81.05345911949685</v>
       </c>
+      <c r="G16" s="3" t="n">
+        <v>8.411949685534591</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1289,6 +1340,9 @@
       <c r="F17" s="3" t="n">
         <v>27.88135593220339</v>
       </c>
+      <c r="G17" s="3" t="n">
+        <v>29.49152542372882</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1311,6 +1365,9 @@
       <c r="F18" s="3" t="n">
         <v>73.11999999999999</v>
       </c>
+      <c r="G18" s="3" t="n">
+        <v>69.67999999999999</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1333,6 +1390,9 @@
       <c r="F19" s="3" t="n">
         <v>40.49382716049383</v>
       </c>
+      <c r="G19" s="3" t="n">
+        <v>40.74074074074074</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1355,6 +1415,9 @@
       <c r="F20" s="3" t="n">
         <v>18.49315068493151</v>
       </c>
+      <c r="G20" s="3" t="n">
+        <v>20.2054794520548</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1376,6 +1439,9 @@
       </c>
       <c r="F21" s="3" t="n">
         <v>65.17241379310344</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>65.05747126436782</v>
       </c>
     </row>
     <row r="22">
@@ -1397,9 +1463,12 @@
       <c r="F22" s="5" t="n">
         <v>47.26318074261048</v>
       </c>
+      <c r="G22" s="5" t="n">
+        <v>43.52004389770321</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F22"/>
+  <autoFilter ref="A1:G22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>